<commit_message>
Fase 1: actualiza entregables y agrega wireframe, presentacion visual y video
- Actualiza documentos grupales (guia definicion proyecto, registro uso IA,
  presentacion) e individuales (autoevaluaciones y diario de reflexion)
- Agrega Wireframe_Chatbot_Soporte_v11.html
- Agrega Presentacion Proyecto (visual).pptx
- Agrega video de recorrido Chatbot-Soporte-Recorrido.mp4

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 1 - Planificación/Grupal/Plantilla Registro Uso IA Capstone.xlsx
+++ b/Fase 1 - Planificación/Grupal/Plantilla Registro Uso IA Capstone.xlsx
@@ -7,7 +7,7 @@
   </sheets>
   <definedNames>
     <definedName name="Z_5ED838EB_82BB_4430_BF98_0EC20343A696_.wvu.FilterData" localSheetId="0" hidden="1">'Registro IA'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registro IA'!$A$1:$L$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registro IA'!$A$1:$L$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="2" min="1" max="1"/>
@@ -1529,10 +1529,440 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="2"/>
-    <row r="22" ht="15.75" customHeight="1" s="2"/>
-    <row r="23" ht="15.75" customHeight="1" s="2"/>
-    <row r="24" ht="15.75" customHeight="1" s="2"/>
+    <row r="18" ht="105" customHeight="1" s="2">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Acotar el alcance de la versión que se defiende y abrir la copia de trabajo del equipo.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Tomando como base el proyecto entregado por la empresa, decidir qué queda dentro de la versión 1 y dejar la decisión documentada, con una copia del código sobre la que el equipo pueda trabajar sin tocar lo recibido.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Carpeta proyecto/ como copia de trabajo, base-alloxentric/ congelada como referencia, y el ADR 0002 que deja WhatsApp fuera de la versión 1. Frontend confirmado en React 18 + Vite.</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Se descartó borrar el código de WhatsApp: los 4 endpoints quedan en el repositorio pero inactivos, para no perder trabajo ya hecho si el alcance se amplía más adelante.</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Verificado con diff -rq que la copia es idéntica al original, y con git status que base-alloxentric/ queda intacta. Se detectó además que la integración continua corría sobre la base congelada en vez de sobre la copia de trabajo, y se corrigió.</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Evita que el equipo modifique la entrega de la empresa y deja por escrito qué se defiende.</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>La decisión de sacar WhatsApp la tomó el equipo; la IA documentó consecuencias y detectó las pantallas que todavía lo ofrecen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="105" customHeight="1" s="2">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Obtener una segunda opinión crítica sobre el wireframe v5 antes de llevarlo a Figma.</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Revisar el wireframe generado en agosto con criterio de diseño de producto y señalar qué está mal resuelto, sin suavizar el diagnóstico.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Revisión escrita con ocho problemas concretos: indicadores con variaciones inventadas, jerarquía plana, tablas sin estados vacíos, iconografía inconsistente y textos de relleno.</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>El equipo pidió expresamente una crítica dura porque el resultado 'se veía muy generado por IA'. Se descartó la primera revisión, que era complaciente.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Cada problema se apoya en un elemento localizable del archivo, no en impresiones generales; se recorrió el wireframe pantalla por pantalla en el navegador.</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Evitó llevar a Figma un diseño que habría que rehacer después.</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Los mockups definitivos son responsabilidad de Manuel Jansen; esta revisión es el insumo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="105" customHeight="1" s="2">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Rediseñar por completo la interfaz del sistema a partir de esa revisión.</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Rehacer el wireframe aplicando las ocho correcciones, con la paleta corporativa real, tres idiomas que traduzcan de verdad y un fondo con movimiento discreto.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Wireframe v11: 12 pantallas, 4 roles, tema claro y oscuro, y un selector ES/EN/PT con las 342 cadenas traducidas.</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Seis iteraciones sobre observaciones del equipo: espaciados, la barra superior que se partía en pantallas angostas, el logotipo que quedaba blanco entero en modo oscuro y un fondo que no dialogaba con la navegación.</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Cada versión se abrió en Chrome sin interfaz y se capturó para revisarla. La traducción se comprobó con un script que repite el mismo recorrido del DOM que hace la página y cuenta las cadenas sin traducir: quedaron en cero.</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Da a Figma un punto de partida ya resuelto en vez de una primera versión que corregir.</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>El logotipo en modo oscuro se resolvió como lo pidió el equipo: el hexágono a todo color y solo el texto en blanco, según la guía de marca de Alloxentric.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="105" customHeight="1" s="2">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Dibujar el modelo de datos y los casos de uso del sistema.</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Generar los dos diagramas en formato editable, leyendo las tablas y las claves foráneas del código real en vez de suponerlas, y con el alcance vigente.</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Los archivos modelo-datos.excalidraw y casos-de-uso.excalidraw, editables en excalidraw.com y exportables para el informe.</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Se reemplazaron los diagramas de agosto, que describían la planificación previa del equipo y no el sistema real. Los casos de uso se ajustaron para no incluir WhatsApp.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Las tablas y relaciones se leyeron de backend/app/models.py, no de la documentación; se verificó que los dos archivos cargan como JSON válido y sin vínculos rotos.</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Cubre dos apartados exigidos por la guía con diagramas que corresponden al código.</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Se editan a mano en Excalidraw; el script solo sirve para rehacerlos desde cero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="105" customHeight="1" s="2">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Rehacer la presentación del examen sobre el archivo de plantilla entregado por la escuela.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Abrir el .pptx de formato oficial, rellenar sus propias láminas hasta 'Tecnologías utilizadas' y eliminar las de la defensa final.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Presentación Proyecto.pptx con 11 láminas construidas sobre la plantilla, incluido el cronograma en el cuadro de Gantt que la propia plantilla trae.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>La primera versión solo copiaba el orden de los temas de la plantilla y la rehacía con diseño propio. El equipo señaló el error y se rehízo abriendo el archivo real.</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Cada lámina se exportó a imagen desde PowerPoint y se revisó a la vista, que es como se detectaron los textos que desbordaban su caja.</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>La presentación entra en el formato exigido sin retoques manuales.</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>El cronograma ocupa dos láminas: doce actividades no caben legibles en una. Son 11 y no 10, y el contenido igual termina donde pidió el profesor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="105" customHeight="1" s="2">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Construir un segundo mazo de presentación para la demo y la defensa.</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>A partir de una plantilla de referencia que gustó al equipo, armar una presentación con el contenido del proyecto, ilustraciones propias y transiciones animadas.</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Presentación Proyecto (visual).pptx, 13 láminas, con una rueda de seis secciones que gira con transición Morph e ilustraciones dibujadas para este proyecto.</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>La primera versión iba sobre fondo azul oscuro. El equipo advirtió que en proyector los colores oscuros se lavan y el texto chico no se lee, y se rehízo entera con fondos claros y un mínimo de 16 pt.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Revisada exportando las láminas a imagen desde PowerPoint. El generador avisa cuando un texto no cabe a 16 pt en vez de encogerlo, para que el problema se vea al generar.</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Da al equipo un mazo presentable sin contratar diseño ni usar bancos de imágenes.</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>No sustituye al entregable oficial, que sigue siendo el de la plantilla de la escuela. Las ilustraciones se dibujan por código, así que no dependen de licencias de terceros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="105" customHeight="1" s="2">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Exequiel Alvarado</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Claude Code (Anthropic)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Producir un video de recorrido por la interfaz para la presentación.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Grabar un recorrido explicado por el wireframe, con entrada de los logotipos, cada pantalla y ventanas que expliquen para qué sirve cada componente.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Video de 1 min 53 s en 1920x1080, con 20 explicaciones sobre las nueve pantallas y música de fondo, incrustado además en el mazo visual.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Se descartó colocar las ventanas explicativas a ojo sobre las capturas: el script mide cada componente en la página real y coloca los recuadros con esas medidas, así que el video se rehace solo cuando cambia el wireframe.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>El audio se midió antes de darlo por bueno: nivel medio, pico y el cierre, donde se detectó que el corte se oía y se alargó el apagado a 3 segundos. El resultado se revisó completo.</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Permite mostrar el sistema en la defensa sin depender de que la demo en vivo funcione.</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>La música es sintetizada para este montaje: dura exactamente lo que el video y no arrastra licencias de terceros.</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="15.75" customHeight="1" s="2"/>
     <row r="26" ht="15.75" customHeight="1" s="2"/>
     <row r="27" ht="15.75" customHeight="1" s="2"/>
@@ -2510,7 +2940,7 @@
     <row r="999" ht="15.75" customHeight="1" s="2"/>
     <row r="1000" ht="15.75" customHeight="1" s="2"/>
   </sheetData>
-  <autoFilter ref="A1:L17"/>
+  <autoFilter ref="A1:L24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <tableParts count="1">

</xml_diff>